<commit_message>
finition formulaire d'inscription + essai javascript pour affichage en fonction des choix
</commit_message>
<xml_diff>
--- a/ressources/emploi_du_temps_des_cours.xlsx
+++ b/ressources/emploi_du_temps_des_cours.xlsx
@@ -313,7 +313,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -382,11 +382,55 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="57">
+  <cellXfs count="89">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -405,113 +449,11 @@
     <xf numFmtId="0" fontId="5" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="11" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="12" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="13" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="14" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="14" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="12" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="15" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="15" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="15" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="16" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="16" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="16" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="17" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="17" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="17" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="14" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top"/>
@@ -519,6 +461,12 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -528,7 +476,109 @@
     <xf numFmtId="0" fontId="3" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="16" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="16" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="16" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="14" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="14" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="14" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="13" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="12" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="12" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="17" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="17" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="17" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="15" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="15" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="15" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -537,20 +587,110 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="16" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="16" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="16" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="17" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="17" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="17" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="13" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="13" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="12" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="12" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="12" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="13" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="15" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="16" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="17" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="12" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="14" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -852,159 +992,159 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:53" s="56" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="49"/>
-      <c r="B2" s="46" t="s">
+    <row r="2" spans="1:53" s="13" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="12"/>
+      <c r="B2" s="14" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="47"/>
-      <c r="D2" s="47"/>
-      <c r="E2" s="48"/>
-      <c r="F2" s="50" t="s">
+      <c r="C2" s="15"/>
+      <c r="D2" s="15"/>
+      <c r="E2" s="16"/>
+      <c r="F2" s="52" t="s">
         <v>8</v>
       </c>
-      <c r="G2" s="50"/>
-      <c r="H2" s="50"/>
-      <c r="I2" s="51"/>
-      <c r="J2" s="52" t="s">
+      <c r="G2" s="52"/>
+      <c r="H2" s="52"/>
+      <c r="I2" s="53"/>
+      <c r="J2" s="49" t="s">
         <v>9</v>
       </c>
-      <c r="K2" s="52"/>
-      <c r="L2" s="52"/>
-      <c r="M2" s="53"/>
-      <c r="N2" s="54" t="s">
+      <c r="K2" s="49"/>
+      <c r="L2" s="49"/>
+      <c r="M2" s="50"/>
+      <c r="N2" s="48" t="s">
         <v>10</v>
       </c>
-      <c r="O2" s="52"/>
-      <c r="P2" s="52"/>
-      <c r="Q2" s="53"/>
-      <c r="R2" s="52" t="s">
+      <c r="O2" s="49"/>
+      <c r="P2" s="49"/>
+      <c r="Q2" s="50"/>
+      <c r="R2" s="49" t="s">
         <v>11</v>
       </c>
-      <c r="S2" s="52"/>
-      <c r="T2" s="52"/>
-      <c r="U2" s="53"/>
-      <c r="V2" s="52" t="s">
+      <c r="S2" s="49"/>
+      <c r="T2" s="49"/>
+      <c r="U2" s="50"/>
+      <c r="V2" s="49" t="s">
         <v>12</v>
       </c>
-      <c r="W2" s="52"/>
-      <c r="X2" s="52"/>
-      <c r="Y2" s="53"/>
-      <c r="Z2" s="52" t="s">
+      <c r="W2" s="49"/>
+      <c r="X2" s="49"/>
+      <c r="Y2" s="50"/>
+      <c r="Z2" s="49" t="s">
         <v>13</v>
       </c>
-      <c r="AA2" s="52"/>
-      <c r="AB2" s="52"/>
-      <c r="AC2" s="53"/>
-      <c r="AD2" s="52" t="s">
+      <c r="AA2" s="49"/>
+      <c r="AB2" s="49"/>
+      <c r="AC2" s="50"/>
+      <c r="AD2" s="49" t="s">
         <v>14</v>
       </c>
-      <c r="AE2" s="52"/>
-      <c r="AF2" s="52"/>
-      <c r="AG2" s="53"/>
-      <c r="AH2" s="52" t="s">
+      <c r="AE2" s="49"/>
+      <c r="AF2" s="49"/>
+      <c r="AG2" s="50"/>
+      <c r="AH2" s="49" t="s">
         <v>15</v>
       </c>
-      <c r="AI2" s="52"/>
-      <c r="AJ2" s="52"/>
-      <c r="AK2" s="53"/>
-      <c r="AL2" s="52" t="s">
+      <c r="AI2" s="49"/>
+      <c r="AJ2" s="49"/>
+      <c r="AK2" s="50"/>
+      <c r="AL2" s="49" t="s">
         <v>16</v>
       </c>
-      <c r="AM2" s="52"/>
-      <c r="AN2" s="52"/>
-      <c r="AO2" s="53"/>
-      <c r="AP2" s="52" t="s">
+      <c r="AM2" s="49"/>
+      <c r="AN2" s="49"/>
+      <c r="AO2" s="50"/>
+      <c r="AP2" s="49" t="s">
         <v>17</v>
       </c>
-      <c r="AQ2" s="52"/>
-      <c r="AR2" s="52"/>
-      <c r="AS2" s="53"/>
-      <c r="AT2" s="54" t="s">
+      <c r="AQ2" s="49"/>
+      <c r="AR2" s="49"/>
+      <c r="AS2" s="50"/>
+      <c r="AT2" s="48" t="s">
         <v>18</v>
       </c>
-      <c r="AU2" s="52"/>
-      <c r="AV2" s="52"/>
-      <c r="AW2" s="53"/>
-      <c r="AX2" s="55"/>
-      <c r="AY2" s="55"/>
-      <c r="AZ2" s="55"/>
-      <c r="BA2" s="55"/>
+      <c r="AU2" s="49"/>
+      <c r="AV2" s="49"/>
+      <c r="AW2" s="50"/>
+      <c r="AX2" s="51"/>
+      <c r="AY2" s="51"/>
+      <c r="AZ2" s="51"/>
+      <c r="BA2" s="51"/>
     </row>
-    <row r="3" spans="1:53" s="45" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="44"/>
-      <c r="B3" s="46" t="s">
+    <row r="3" spans="1:53" s="11" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="10"/>
+      <c r="B3" s="14" t="s">
         <v>34</v>
       </c>
-      <c r="C3" s="47"/>
-      <c r="D3" s="47"/>
-      <c r="E3" s="48"/>
-      <c r="F3" s="46" t="s">
+      <c r="C3" s="15"/>
+      <c r="D3" s="15"/>
+      <c r="E3" s="16"/>
+      <c r="F3" s="14" t="s">
         <v>34</v>
       </c>
-      <c r="G3" s="47"/>
-      <c r="H3" s="47"/>
-      <c r="I3" s="48"/>
-      <c r="J3" s="46" t="s">
+      <c r="G3" s="15"/>
+      <c r="H3" s="15"/>
+      <c r="I3" s="16"/>
+      <c r="J3" s="14" t="s">
         <v>34</v>
       </c>
-      <c r="K3" s="47"/>
-      <c r="L3" s="47"/>
-      <c r="M3" s="48"/>
-      <c r="N3" s="46" t="s">
+      <c r="K3" s="15"/>
+      <c r="L3" s="15"/>
+      <c r="M3" s="16"/>
+      <c r="N3" s="14" t="s">
         <v>34</v>
       </c>
-      <c r="O3" s="47"/>
-      <c r="P3" s="47"/>
-      <c r="Q3" s="48"/>
-      <c r="R3" s="46" t="s">
+      <c r="O3" s="15"/>
+      <c r="P3" s="15"/>
+      <c r="Q3" s="16"/>
+      <c r="R3" s="14" t="s">
         <v>34</v>
       </c>
-      <c r="S3" s="47"/>
-      <c r="T3" s="47"/>
-      <c r="U3" s="48"/>
-      <c r="V3" s="46" t="s">
+      <c r="S3" s="15"/>
+      <c r="T3" s="15"/>
+      <c r="U3" s="16"/>
+      <c r="V3" s="14" t="s">
         <v>34</v>
       </c>
-      <c r="W3" s="47"/>
-      <c r="X3" s="47"/>
-      <c r="Y3" s="48"/>
-      <c r="Z3" s="46" t="s">
+      <c r="W3" s="15"/>
+      <c r="X3" s="15"/>
+      <c r="Y3" s="16"/>
+      <c r="Z3" s="14" t="s">
         <v>34</v>
       </c>
-      <c r="AA3" s="47"/>
-      <c r="AB3" s="47"/>
-      <c r="AC3" s="48"/>
-      <c r="AD3" s="46" t="s">
+      <c r="AA3" s="15"/>
+      <c r="AB3" s="15"/>
+      <c r="AC3" s="16"/>
+      <c r="AD3" s="14" t="s">
         <v>34</v>
       </c>
-      <c r="AE3" s="47"/>
-      <c r="AF3" s="47"/>
-      <c r="AG3" s="48"/>
-      <c r="AH3" s="46" t="s">
+      <c r="AE3" s="15"/>
+      <c r="AF3" s="15"/>
+      <c r="AG3" s="16"/>
+      <c r="AH3" s="14" t="s">
         <v>34</v>
       </c>
-      <c r="AI3" s="47"/>
-      <c r="AJ3" s="47"/>
-      <c r="AK3" s="48"/>
-      <c r="AL3" s="46" t="s">
+      <c r="AI3" s="15"/>
+      <c r="AJ3" s="15"/>
+      <c r="AK3" s="16"/>
+      <c r="AL3" s="14" t="s">
         <v>34</v>
       </c>
-      <c r="AM3" s="47"/>
-      <c r="AN3" s="47"/>
-      <c r="AO3" s="48"/>
-      <c r="AP3" s="46" t="s">
+      <c r="AM3" s="15"/>
+      <c r="AN3" s="15"/>
+      <c r="AO3" s="16"/>
+      <c r="AP3" s="14" t="s">
         <v>34</v>
       </c>
-      <c r="AQ3" s="47"/>
-      <c r="AR3" s="47"/>
-      <c r="AS3" s="48"/>
-      <c r="AT3" s="46" t="s">
+      <c r="AQ3" s="15"/>
+      <c r="AR3" s="15"/>
+      <c r="AS3" s="16"/>
+      <c r="AT3" s="14" t="s">
         <v>34</v>
       </c>
-      <c r="AU3" s="47"/>
-      <c r="AV3" s="47"/>
-      <c r="AW3" s="48"/>
+      <c r="AU3" s="15"/>
+      <c r="AV3" s="15"/>
+      <c r="AW3" s="16"/>
     </row>
     <row r="4" spans="1:53" s="4" customFormat="1" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A4" s="5" t="s">
@@ -1018,62 +1158,62 @@
       <c r="G4" s="6"/>
       <c r="H4" s="6"/>
       <c r="I4" s="6"/>
-      <c r="J4" s="9"/>
-      <c r="K4" s="9"/>
-      <c r="L4" s="9"/>
-      <c r="M4" s="9"/>
-      <c r="N4" s="8" t="s">
+      <c r="J4" s="8"/>
+      <c r="K4" s="8"/>
+      <c r="L4" s="8"/>
+      <c r="M4" s="8"/>
+      <c r="N4" s="38" t="s">
         <v>23</v>
       </c>
-      <c r="O4" s="8"/>
-      <c r="P4" s="8"/>
-      <c r="Q4" s="8"/>
-      <c r="R4" s="13" t="s">
+      <c r="O4" s="38"/>
+      <c r="P4" s="38"/>
+      <c r="Q4" s="38"/>
+      <c r="R4" s="39" t="s">
         <v>24</v>
       </c>
-      <c r="S4" s="13"/>
-      <c r="T4" s="13"/>
-      <c r="U4" s="13"/>
-      <c r="V4" s="9"/>
-      <c r="W4" s="9"/>
-      <c r="X4" s="9"/>
-      <c r="Y4" s="9"/>
-      <c r="Z4" s="9"/>
-      <c r="AA4" s="9"/>
-      <c r="AB4" s="9"/>
-      <c r="AC4" s="9"/>
-      <c r="AD4" s="9"/>
-      <c r="AE4" s="9"/>
-      <c r="AF4" s="27" t="s">
+      <c r="S4" s="39"/>
+      <c r="T4" s="39"/>
+      <c r="U4" s="39"/>
+      <c r="V4" s="8"/>
+      <c r="W4" s="8"/>
+      <c r="X4" s="8"/>
+      <c r="Y4" s="8"/>
+      <c r="Z4" s="8"/>
+      <c r="AA4" s="8"/>
+      <c r="AB4" s="8"/>
+      <c r="AC4" s="8"/>
+      <c r="AD4" s="8"/>
+      <c r="AE4" s="8"/>
+      <c r="AF4" s="28" t="s">
         <v>26</v>
       </c>
-      <c r="AG4" s="28"/>
-      <c r="AH4" s="29" t="s">
+      <c r="AG4" s="29"/>
+      <c r="AH4" s="36" t="s">
         <v>27</v>
       </c>
-      <c r="AI4" s="30"/>
-      <c r="AJ4" s="32" t="s">
+      <c r="AI4" s="37"/>
+      <c r="AJ4" s="41" t="s">
         <v>28</v>
       </c>
-      <c r="AK4" s="33"/>
-      <c r="AL4" s="34"/>
-      <c r="AM4" s="35" t="s">
+      <c r="AK4" s="42"/>
+      <c r="AL4" s="43"/>
+      <c r="AM4" s="17" t="s">
         <v>29</v>
       </c>
-      <c r="AN4" s="36"/>
-      <c r="AO4" s="37"/>
-      <c r="AP4" s="21" t="s">
+      <c r="AN4" s="18"/>
+      <c r="AO4" s="19"/>
+      <c r="AP4" s="25" t="s">
         <v>32</v>
       </c>
-      <c r="AQ4" s="31"/>
-      <c r="AR4" s="31"/>
-      <c r="AS4" s="22"/>
-      <c r="AT4" s="12" t="s">
+      <c r="AQ4" s="26"/>
+      <c r="AR4" s="26"/>
+      <c r="AS4" s="27"/>
+      <c r="AT4" s="40" t="s">
         <v>25</v>
       </c>
-      <c r="AU4" s="12"/>
-      <c r="AV4" s="12"/>
-      <c r="AW4" s="10"/>
+      <c r="AU4" s="40"/>
+      <c r="AV4" s="40"/>
+      <c r="AW4" s="9"/>
     </row>
     <row r="5" spans="1:53" s="4" customFormat="1" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="5" t="s">
@@ -1087,143 +1227,143 @@
       <c r="G5" s="6"/>
       <c r="H5" s="6"/>
       <c r="I5" s="6"/>
-      <c r="J5" s="9"/>
-      <c r="K5" s="9"/>
-      <c r="L5" s="9"/>
-      <c r="M5" s="9"/>
-      <c r="N5" s="12" t="s">
+      <c r="J5" s="8"/>
+      <c r="K5" s="8"/>
+      <c r="L5" s="8"/>
+      <c r="M5" s="8"/>
+      <c r="N5" s="40" t="s">
         <v>25</v>
       </c>
-      <c r="O5" s="12"/>
-      <c r="P5" s="12"/>
-      <c r="Q5" s="8" t="s">
+      <c r="O5" s="40"/>
+      <c r="P5" s="40"/>
+      <c r="Q5" s="38" t="s">
         <v>23</v>
       </c>
-      <c r="R5" s="8"/>
-      <c r="S5" s="8"/>
-      <c r="T5" s="8"/>
-      <c r="U5" s="9"/>
-      <c r="V5" s="9"/>
-      <c r="W5" s="9"/>
-      <c r="X5" s="9"/>
-      <c r="Y5" s="9"/>
-      <c r="Z5" s="9"/>
-      <c r="AA5" s="9"/>
-      <c r="AB5" s="9"/>
-      <c r="AC5" s="9"/>
-      <c r="AD5" s="9"/>
-      <c r="AE5" s="9"/>
-      <c r="AF5" s="29" t="s">
+      <c r="R5" s="38"/>
+      <c r="S5" s="38"/>
+      <c r="T5" s="38"/>
+      <c r="U5" s="8"/>
+      <c r="V5" s="8"/>
+      <c r="W5" s="8"/>
+      <c r="X5" s="8"/>
+      <c r="Y5" s="8"/>
+      <c r="Z5" s="8"/>
+      <c r="AA5" s="8"/>
+      <c r="AB5" s="8"/>
+      <c r="AC5" s="8"/>
+      <c r="AD5" s="8"/>
+      <c r="AE5" s="8"/>
+      <c r="AF5" s="36" t="s">
         <v>27</v>
       </c>
-      <c r="AG5" s="30"/>
-      <c r="AH5" s="32" t="s">
+      <c r="AG5" s="37"/>
+      <c r="AH5" s="41" t="s">
         <v>28</v>
       </c>
-      <c r="AI5" s="33"/>
-      <c r="AJ5" s="34"/>
-      <c r="AK5" s="35" t="s">
+      <c r="AI5" s="42"/>
+      <c r="AJ5" s="43"/>
+      <c r="AK5" s="17" t="s">
         <v>29</v>
       </c>
-      <c r="AL5" s="36"/>
-      <c r="AM5" s="37"/>
-      <c r="AN5" s="25" t="s">
+      <c r="AL5" s="18"/>
+      <c r="AM5" s="19"/>
+      <c r="AN5" s="20" t="s">
         <v>33</v>
       </c>
-      <c r="AO5" s="41"/>
-      <c r="AP5" s="41"/>
-      <c r="AQ5" s="26"/>
-      <c r="AR5" s="14" t="s">
+      <c r="AO5" s="21"/>
+      <c r="AP5" s="21"/>
+      <c r="AQ5" s="22"/>
+      <c r="AR5" s="33" t="s">
         <v>24</v>
       </c>
-      <c r="AS5" s="15"/>
-      <c r="AT5" s="15"/>
-      <c r="AU5" s="16"/>
-      <c r="AV5" s="9"/>
-      <c r="AW5" s="9"/>
+      <c r="AS5" s="34"/>
+      <c r="AT5" s="34"/>
+      <c r="AU5" s="35"/>
+      <c r="AV5" s="8"/>
+      <c r="AW5" s="8"/>
     </row>
     <row r="6" spans="1:53" s="4" customFormat="1" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A6" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="17" t="s">
+      <c r="B6" s="47" t="s">
         <v>20</v>
       </c>
-      <c r="C6" s="17"/>
-      <c r="D6" s="18" t="s">
+      <c r="C6" s="47"/>
+      <c r="D6" s="44" t="s">
         <v>19</v>
       </c>
-      <c r="E6" s="18"/>
-      <c r="F6" s="19" t="s">
+      <c r="E6" s="44"/>
+      <c r="F6" s="45" t="s">
         <v>21</v>
       </c>
-      <c r="G6" s="19"/>
-      <c r="H6" s="20" t="s">
+      <c r="G6" s="45"/>
+      <c r="H6" s="46" t="s">
         <v>22</v>
       </c>
-      <c r="I6" s="20"/>
+      <c r="I6" s="46"/>
       <c r="J6" s="23" t="s">
         <v>30</v>
       </c>
       <c r="K6" s="24"/>
-      <c r="L6" s="27" t="s">
+      <c r="L6" s="28" t="s">
         <v>26</v>
       </c>
-      <c r="M6" s="28"/>
-      <c r="N6" s="29" t="s">
+      <c r="M6" s="29"/>
+      <c r="N6" s="36" t="s">
         <v>27</v>
       </c>
-      <c r="O6" s="30"/>
-      <c r="P6" s="9"/>
-      <c r="Q6" s="9"/>
-      <c r="R6" s="9"/>
-      <c r="S6" s="9"/>
-      <c r="T6" s="32" t="s">
+      <c r="O6" s="37"/>
+      <c r="P6" s="8"/>
+      <c r="Q6" s="8"/>
+      <c r="R6" s="8"/>
+      <c r="S6" s="8"/>
+      <c r="T6" s="41" t="s">
         <v>28</v>
       </c>
-      <c r="U6" s="33"/>
-      <c r="V6" s="34"/>
-      <c r="W6" s="35" t="s">
+      <c r="U6" s="42"/>
+      <c r="V6" s="43"/>
+      <c r="W6" s="17" t="s">
         <v>29</v>
       </c>
-      <c r="X6" s="36"/>
-      <c r="Y6" s="37"/>
-      <c r="Z6" s="38" t="s">
+      <c r="X6" s="18"/>
+      <c r="Y6" s="19"/>
+      <c r="Z6" s="30" t="s">
         <v>31</v>
       </c>
-      <c r="AA6" s="39"/>
-      <c r="AB6" s="40"/>
-      <c r="AC6" s="21" t="s">
+      <c r="AA6" s="31"/>
+      <c r="AB6" s="32"/>
+      <c r="AC6" s="25" t="s">
         <v>32</v>
       </c>
-      <c r="AD6" s="31"/>
-      <c r="AE6" s="31"/>
-      <c r="AF6" s="22"/>
-      <c r="AG6" s="43"/>
-      <c r="AH6" s="11"/>
-      <c r="AI6" s="25" t="s">
+      <c r="AD6" s="26"/>
+      <c r="AE6" s="26"/>
+      <c r="AF6" s="27"/>
+      <c r="AG6" s="55"/>
+      <c r="AH6" s="55"/>
+      <c r="AI6" s="20" t="s">
         <v>33</v>
       </c>
-      <c r="AJ6" s="41"/>
-      <c r="AK6" s="41"/>
-      <c r="AL6" s="26"/>
-      <c r="AM6" s="12" t="s">
+      <c r="AJ6" s="21"/>
+      <c r="AK6" s="21"/>
+      <c r="AL6" s="22"/>
+      <c r="AM6" s="40" t="s">
         <v>25</v>
       </c>
-      <c r="AN6" s="12"/>
-      <c r="AO6" s="12"/>
-      <c r="AP6" s="13" t="s">
+      <c r="AN6" s="40"/>
+      <c r="AO6" s="40"/>
+      <c r="AP6" s="39" t="s">
         <v>24</v>
       </c>
-      <c r="AQ6" s="13"/>
-      <c r="AR6" s="13"/>
-      <c r="AS6" s="13"/>
-      <c r="AT6" s="8" t="s">
+      <c r="AQ6" s="39"/>
+      <c r="AR6" s="39"/>
+      <c r="AS6" s="39"/>
+      <c r="AT6" s="38" t="s">
         <v>23</v>
       </c>
-      <c r="AU6" s="8"/>
-      <c r="AV6" s="8"/>
-      <c r="AW6" s="8"/>
+      <c r="AU6" s="38"/>
+      <c r="AV6" s="38"/>
+      <c r="AW6" s="38"/>
     </row>
     <row r="7" spans="1:53" s="4" customFormat="1" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="s">
@@ -1237,260 +1377,246 @@
       <c r="G7" s="6"/>
       <c r="H7" s="6"/>
       <c r="I7" s="6"/>
-      <c r="J7" s="9"/>
-      <c r="K7" s="9"/>
-      <c r="L7" s="9"/>
-      <c r="M7" s="9"/>
-      <c r="N7" s="13" t="s">
+      <c r="J7" s="8"/>
+      <c r="K7" s="8"/>
+      <c r="L7" s="8"/>
+      <c r="M7" s="8"/>
+      <c r="N7" s="39" t="s">
         <v>24</v>
       </c>
-      <c r="O7" s="13"/>
-      <c r="P7" s="13"/>
-      <c r="Q7" s="13"/>
-      <c r="R7" s="8" t="s">
+      <c r="O7" s="39"/>
+      <c r="P7" s="39"/>
+      <c r="Q7" s="39"/>
+      <c r="R7" s="38" t="s">
         <v>23</v>
       </c>
-      <c r="S7" s="8"/>
-      <c r="T7" s="8"/>
-      <c r="U7" s="8"/>
-      <c r="V7" s="9"/>
-      <c r="W7" s="9"/>
-      <c r="X7" s="9"/>
-      <c r="Y7" s="9"/>
-      <c r="Z7" s="9"/>
-      <c r="AA7" s="9"/>
-      <c r="AB7" s="9"/>
-      <c r="AC7" s="9"/>
-      <c r="AD7" s="9"/>
-      <c r="AE7" s="9"/>
-      <c r="AF7" s="32" t="s">
+      <c r="S7" s="38"/>
+      <c r="T7" s="38"/>
+      <c r="U7" s="38"/>
+      <c r="V7" s="8"/>
+      <c r="W7" s="8"/>
+      <c r="X7" s="8"/>
+      <c r="Y7" s="8"/>
+      <c r="Z7" s="8"/>
+      <c r="AA7" s="8"/>
+      <c r="AB7" s="8"/>
+      <c r="AC7" s="8"/>
+      <c r="AD7" s="8"/>
+      <c r="AE7" s="8"/>
+      <c r="AF7" s="41" t="s">
         <v>28</v>
       </c>
-      <c r="AG7" s="33"/>
-      <c r="AH7" s="34"/>
-      <c r="AI7" s="35" t="s">
+      <c r="AG7" s="42"/>
+      <c r="AH7" s="43"/>
+      <c r="AI7" s="17" t="s">
         <v>29</v>
       </c>
-      <c r="AJ7" s="36"/>
-      <c r="AK7" s="37"/>
-      <c r="AL7" s="38" t="s">
+      <c r="AJ7" s="18"/>
+      <c r="AK7" s="19"/>
+      <c r="AL7" s="30" t="s">
         <v>31</v>
       </c>
-      <c r="AM7" s="39"/>
-      <c r="AN7" s="40"/>
-      <c r="AO7" s="29" t="s">
+      <c r="AM7" s="31"/>
+      <c r="AN7" s="32"/>
+      <c r="AO7" s="36" t="s">
         <v>27</v>
       </c>
-      <c r="AP7" s="30"/>
-      <c r="AQ7" s="27" t="s">
+      <c r="AP7" s="37"/>
+      <c r="AQ7" s="28" t="s">
         <v>26</v>
       </c>
-      <c r="AR7" s="28"/>
-      <c r="AS7" s="9"/>
-      <c r="AT7" s="9"/>
-      <c r="AU7" s="12" t="s">
+      <c r="AR7" s="29"/>
+      <c r="AS7" s="86" t="s">
         <v>25</v>
       </c>
-      <c r="AV7" s="12"/>
-      <c r="AW7" s="12"/>
+      <c r="AT7" s="87"/>
+      <c r="AU7" s="88"/>
+      <c r="AV7" s="54"/>
+      <c r="AW7" s="54"/>
     </row>
     <row r="8" spans="1:53" s="4" customFormat="1" ht="13.8" x14ac:dyDescent="0.3">
-      <c r="A8" s="5" t="s">
+      <c r="A8" s="56" t="s">
         <v>5</v>
       </c>
-      <c r="B8" s="7"/>
-      <c r="C8" s="7"/>
-      <c r="D8" s="7"/>
-      <c r="E8" s="7"/>
-      <c r="F8" s="6"/>
-      <c r="G8" s="6"/>
-      <c r="H8" s="6"/>
-      <c r="I8" s="6"/>
-      <c r="J8" s="9"/>
-      <c r="K8" s="9"/>
-      <c r="L8" s="9"/>
-      <c r="M8" s="9"/>
-      <c r="N8" s="12" t="s">
+      <c r="B8" s="57"/>
+      <c r="C8" s="57"/>
+      <c r="D8" s="57"/>
+      <c r="E8" s="57"/>
+      <c r="F8" s="58"/>
+      <c r="G8" s="58"/>
+      <c r="H8" s="58"/>
+      <c r="I8" s="58"/>
+      <c r="J8" s="59"/>
+      <c r="K8" s="59"/>
+      <c r="L8" s="59"/>
+      <c r="M8" s="59"/>
+      <c r="N8" s="60" t="s">
         <v>25</v>
       </c>
-      <c r="O8" s="12"/>
-      <c r="P8" s="12"/>
-      <c r="Q8" s="13" t="s">
+      <c r="O8" s="60"/>
+      <c r="P8" s="60"/>
+      <c r="Q8" s="61" t="s">
         <v>24</v>
       </c>
-      <c r="R8" s="13"/>
-      <c r="S8" s="13"/>
-      <c r="T8" s="13"/>
-      <c r="U8" s="9"/>
-      <c r="V8" s="9"/>
-      <c r="W8" s="9"/>
-      <c r="X8" s="9"/>
-      <c r="Y8" s="9"/>
-      <c r="Z8" s="9"/>
-      <c r="AA8" s="9"/>
-      <c r="AB8" s="9"/>
-      <c r="AC8" s="9"/>
-      <c r="AD8" s="9"/>
-      <c r="AE8" s="42"/>
-      <c r="AF8" s="35" t="s">
+      <c r="R8" s="61"/>
+      <c r="S8" s="61"/>
+      <c r="T8" s="61"/>
+      <c r="U8" s="59"/>
+      <c r="V8" s="59"/>
+      <c r="W8" s="59"/>
+      <c r="X8" s="59"/>
+      <c r="Y8" s="59"/>
+      <c r="Z8" s="59"/>
+      <c r="AA8" s="59"/>
+      <c r="AB8" s="59"/>
+      <c r="AC8" s="59"/>
+      <c r="AD8" s="59"/>
+      <c r="AE8" s="62"/>
+      <c r="AF8" s="63" t="s">
         <v>29</v>
       </c>
-      <c r="AG8" s="36"/>
-      <c r="AH8" s="37"/>
-      <c r="AI8" s="38" t="s">
+      <c r="AG8" s="64"/>
+      <c r="AH8" s="65"/>
+      <c r="AI8" s="66" t="s">
         <v>31</v>
       </c>
-      <c r="AJ8" s="39"/>
-      <c r="AK8" s="40"/>
-      <c r="AL8" s="27" t="s">
+      <c r="AJ8" s="67"/>
+      <c r="AK8" s="68"/>
+      <c r="AL8" s="69" t="s">
         <v>26</v>
       </c>
-      <c r="AM8" s="28"/>
-      <c r="AN8" s="23" t="s">
+      <c r="AM8" s="70"/>
+      <c r="AN8" s="71" t="s">
         <v>30</v>
       </c>
-      <c r="AO8" s="24"/>
-      <c r="AP8" s="21" t="s">
+      <c r="AO8" s="72"/>
+      <c r="AP8" s="73" t="s">
         <v>32</v>
       </c>
-      <c r="AQ8" s="31"/>
-      <c r="AR8" s="31"/>
-      <c r="AS8" s="22"/>
-      <c r="AT8" s="8" t="s">
+      <c r="AQ8" s="74"/>
+      <c r="AR8" s="74"/>
+      <c r="AS8" s="75"/>
+      <c r="AT8" s="76" t="s">
         <v>23</v>
       </c>
-      <c r="AU8" s="8"/>
-      <c r="AV8" s="8"/>
-      <c r="AW8" s="8"/>
+      <c r="AU8" s="76"/>
+      <c r="AV8" s="76"/>
+      <c r="AW8" s="76"/>
     </row>
-    <row r="9" spans="1:53" s="4" customFormat="1" ht="13.8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:53" s="85" customFormat="1" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A9" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="B9" s="17" t="s">
+      <c r="B9" s="47" t="s">
         <v>20</v>
       </c>
-      <c r="C9" s="17"/>
-      <c r="D9" s="18" t="s">
+      <c r="C9" s="47"/>
+      <c r="D9" s="44" t="s">
         <v>19</v>
       </c>
-      <c r="E9" s="18"/>
-      <c r="F9" s="19" t="s">
+      <c r="E9" s="44"/>
+      <c r="F9" s="45" t="s">
         <v>21</v>
       </c>
-      <c r="G9" s="19"/>
-      <c r="H9" s="20" t="s">
+      <c r="G9" s="45"/>
+      <c r="H9" s="46" t="s">
         <v>22</v>
       </c>
-      <c r="I9" s="20"/>
-      <c r="J9" s="23" t="s">
+      <c r="I9" s="46"/>
+      <c r="J9" s="77" t="s">
         <v>30</v>
       </c>
-      <c r="K9" s="24"/>
-      <c r="L9" s="27" t="s">
+      <c r="K9" s="77"/>
+      <c r="L9" s="78" t="s">
         <v>26</v>
       </c>
-      <c r="M9" s="28"/>
-      <c r="N9" s="29" t="s">
+      <c r="M9" s="78"/>
+      <c r="N9" s="79" t="s">
         <v>27</v>
       </c>
-      <c r="O9" s="30"/>
-      <c r="P9" s="9"/>
-      <c r="Q9" s="9"/>
-      <c r="R9" s="9"/>
-      <c r="S9" s="9"/>
-      <c r="T9" s="32" t="s">
+      <c r="O9" s="79"/>
+      <c r="P9" s="8"/>
+      <c r="Q9" s="8"/>
+      <c r="R9" s="8"/>
+      <c r="S9" s="8"/>
+      <c r="T9" s="80" t="s">
         <v>28</v>
       </c>
-      <c r="U9" s="33"/>
-      <c r="V9" s="34"/>
-      <c r="W9" s="35" t="s">
+      <c r="U9" s="80"/>
+      <c r="V9" s="80"/>
+      <c r="W9" s="81" t="s">
         <v>29</v>
       </c>
-      <c r="X9" s="36"/>
-      <c r="Y9" s="37"/>
-      <c r="Z9" s="38" t="s">
+      <c r="X9" s="81"/>
+      <c r="Y9" s="81"/>
+      <c r="Z9" s="82" t="s">
         <v>31</v>
       </c>
-      <c r="AA9" s="39"/>
-      <c r="AB9" s="40"/>
-      <c r="AC9" s="21" t="s">
+      <c r="AA9" s="82"/>
+      <c r="AB9" s="82"/>
+      <c r="AC9" s="83" t="s">
         <v>32</v>
       </c>
-      <c r="AD9" s="31"/>
-      <c r="AE9" s="31"/>
-      <c r="AF9" s="22"/>
-      <c r="AG9" s="43"/>
-      <c r="AH9" s="11"/>
-      <c r="AI9" s="25" t="s">
+      <c r="AD9" s="83"/>
+      <c r="AE9" s="83"/>
+      <c r="AF9" s="83"/>
+      <c r="AG9" s="55"/>
+      <c r="AH9" s="55"/>
+      <c r="AI9" s="84" t="s">
         <v>33</v>
       </c>
-      <c r="AJ9" s="41"/>
-      <c r="AK9" s="41"/>
-      <c r="AL9" s="26"/>
-      <c r="AM9" s="8" t="s">
+      <c r="AJ9" s="84"/>
+      <c r="AK9" s="84"/>
+      <c r="AL9" s="84"/>
+      <c r="AM9" s="38" t="s">
         <v>23</v>
       </c>
-      <c r="AN9" s="8"/>
-      <c r="AO9" s="8"/>
-      <c r="AP9" s="8"/>
-      <c r="AQ9" s="13" t="s">
+      <c r="AN9" s="38"/>
+      <c r="AO9" s="38"/>
+      <c r="AP9" s="38"/>
+      <c r="AQ9" s="39" t="s">
         <v>24</v>
       </c>
-      <c r="AR9" s="13"/>
-      <c r="AS9" s="13"/>
-      <c r="AT9" s="13"/>
-      <c r="AU9" s="12" t="s">
+      <c r="AR9" s="39"/>
+      <c r="AS9" s="39"/>
+      <c r="AT9" s="39"/>
+      <c r="AU9" s="40" t="s">
         <v>25</v>
       </c>
-      <c r="AV9" s="12"/>
-      <c r="AW9" s="12"/>
+      <c r="AV9" s="40"/>
+      <c r="AW9" s="40"/>
     </row>
   </sheetData>
   <mergeCells count="86">
-    <mergeCell ref="AD3:AG3"/>
-    <mergeCell ref="AH3:AK3"/>
-    <mergeCell ref="AL3:AO3"/>
-    <mergeCell ref="AP3:AS3"/>
-    <mergeCell ref="AF8:AH8"/>
-    <mergeCell ref="AI6:AL6"/>
-    <mergeCell ref="AI9:AL9"/>
-    <mergeCell ref="F3:I3"/>
-    <mergeCell ref="J3:M3"/>
-    <mergeCell ref="N3:Q3"/>
-    <mergeCell ref="R3:U3"/>
-    <mergeCell ref="V3:Y3"/>
-    <mergeCell ref="Z3:AC3"/>
-    <mergeCell ref="AN8:AO8"/>
-    <mergeCell ref="AP8:AS8"/>
-    <mergeCell ref="AL8:AM8"/>
-    <mergeCell ref="AI8:AK8"/>
-    <mergeCell ref="AK5:AM5"/>
-    <mergeCell ref="AN5:AQ5"/>
-    <mergeCell ref="AR5:AU5"/>
-    <mergeCell ref="AL7:AN7"/>
-    <mergeCell ref="AO7:AP7"/>
-    <mergeCell ref="AQ7:AR7"/>
-    <mergeCell ref="AC9:AF9"/>
-    <mergeCell ref="AM9:AP9"/>
-    <mergeCell ref="AQ9:AT9"/>
-    <mergeCell ref="AU9:AW9"/>
-    <mergeCell ref="AH4:AI4"/>
-    <mergeCell ref="AH5:AJ5"/>
-    <mergeCell ref="AI7:AK7"/>
-    <mergeCell ref="AJ4:AL4"/>
-    <mergeCell ref="AC6:AF6"/>
-    <mergeCell ref="AT6:AW6"/>
-    <mergeCell ref="AP6:AS6"/>
-    <mergeCell ref="AM6:AO6"/>
-    <mergeCell ref="L9:M9"/>
-    <mergeCell ref="N9:O9"/>
-    <mergeCell ref="T9:V9"/>
-    <mergeCell ref="W9:Y9"/>
-    <mergeCell ref="Z9:AB9"/>
-    <mergeCell ref="D9:E9"/>
-    <mergeCell ref="F9:G9"/>
-    <mergeCell ref="H9:I9"/>
+    <mergeCell ref="R2:U2"/>
+    <mergeCell ref="AS7:AU7"/>
+    <mergeCell ref="B3:E3"/>
+    <mergeCell ref="B2:E2"/>
+    <mergeCell ref="F2:I2"/>
+    <mergeCell ref="J2:M2"/>
+    <mergeCell ref="N2:Q2"/>
+    <mergeCell ref="V2:Y2"/>
+    <mergeCell ref="Z2:AC2"/>
+    <mergeCell ref="AD2:AG2"/>
+    <mergeCell ref="AH2:AK2"/>
+    <mergeCell ref="AL2:AO2"/>
+    <mergeCell ref="AT2:AW2"/>
+    <mergeCell ref="AX2:BA2"/>
+    <mergeCell ref="AT3:AW3"/>
+    <mergeCell ref="AM4:AO4"/>
+    <mergeCell ref="AP4:AS4"/>
+    <mergeCell ref="AT4:AV4"/>
+    <mergeCell ref="AP2:AS2"/>
+    <mergeCell ref="N4:Q4"/>
+    <mergeCell ref="N7:Q7"/>
+    <mergeCell ref="R4:U4"/>
+    <mergeCell ref="R7:U7"/>
+    <mergeCell ref="N5:P5"/>
+    <mergeCell ref="Q5:T5"/>
+    <mergeCell ref="N8:P8"/>
+    <mergeCell ref="Q8:T8"/>
+    <mergeCell ref="AT8:AW8"/>
+    <mergeCell ref="AF5:AG5"/>
     <mergeCell ref="J6:K6"/>
     <mergeCell ref="J9:K9"/>
     <mergeCell ref="L6:M6"/>
@@ -1503,37 +1629,51 @@
     <mergeCell ref="T6:V6"/>
     <mergeCell ref="W6:Y6"/>
     <mergeCell ref="Z6:AB6"/>
-    <mergeCell ref="Q5:T5"/>
-    <mergeCell ref="AU7:AW7"/>
-    <mergeCell ref="N8:P8"/>
-    <mergeCell ref="Q8:T8"/>
-    <mergeCell ref="AT8:AW8"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="T9:V9"/>
+    <mergeCell ref="W9:Y9"/>
+    <mergeCell ref="Z9:AB9"/>
+    <mergeCell ref="D9:E9"/>
+    <mergeCell ref="F9:G9"/>
+    <mergeCell ref="H9:I9"/>
+    <mergeCell ref="AQ9:AT9"/>
+    <mergeCell ref="AU9:AW9"/>
+    <mergeCell ref="AH4:AI4"/>
+    <mergeCell ref="AH5:AJ5"/>
+    <mergeCell ref="AI7:AK7"/>
+    <mergeCell ref="AJ4:AL4"/>
+    <mergeCell ref="AT6:AW6"/>
+    <mergeCell ref="AP6:AS6"/>
+    <mergeCell ref="AM6:AO6"/>
+    <mergeCell ref="AI9:AL9"/>
+    <mergeCell ref="F3:I3"/>
+    <mergeCell ref="J3:M3"/>
+    <mergeCell ref="N3:Q3"/>
+    <mergeCell ref="R3:U3"/>
+    <mergeCell ref="V3:Y3"/>
+    <mergeCell ref="Z3:AC3"/>
+    <mergeCell ref="AL8:AM8"/>
+    <mergeCell ref="AI8:AK8"/>
+    <mergeCell ref="AK5:AM5"/>
+    <mergeCell ref="AL7:AN7"/>
+    <mergeCell ref="AC9:AF9"/>
+    <mergeCell ref="AM9:AP9"/>
+    <mergeCell ref="AC6:AF6"/>
+    <mergeCell ref="L9:M9"/>
+    <mergeCell ref="N9:O9"/>
+    <mergeCell ref="AD3:AG3"/>
+    <mergeCell ref="AH3:AK3"/>
+    <mergeCell ref="AL3:AO3"/>
+    <mergeCell ref="AP3:AS3"/>
+    <mergeCell ref="AF8:AH8"/>
+    <mergeCell ref="AI6:AL6"/>
+    <mergeCell ref="AN8:AO8"/>
+    <mergeCell ref="AP8:AS8"/>
+    <mergeCell ref="AN5:AQ5"/>
+    <mergeCell ref="AR5:AU5"/>
+    <mergeCell ref="AO7:AP7"/>
+    <mergeCell ref="AQ7:AR7"/>
     <mergeCell ref="AF4:AG4"/>
-    <mergeCell ref="AF5:AG5"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="N4:Q4"/>
-    <mergeCell ref="N7:Q7"/>
-    <mergeCell ref="R4:U4"/>
-    <mergeCell ref="R7:U7"/>
-    <mergeCell ref="N5:P5"/>
-    <mergeCell ref="AT2:AW2"/>
-    <mergeCell ref="AX2:BA2"/>
-    <mergeCell ref="AT3:AW3"/>
-    <mergeCell ref="AM4:AO4"/>
-    <mergeCell ref="AP4:AS4"/>
-    <mergeCell ref="AT4:AV4"/>
-    <mergeCell ref="V2:Y2"/>
-    <mergeCell ref="Z2:AC2"/>
-    <mergeCell ref="AD2:AG2"/>
-    <mergeCell ref="AH2:AK2"/>
-    <mergeCell ref="AL2:AO2"/>
-    <mergeCell ref="AP2:AS2"/>
-    <mergeCell ref="B3:E3"/>
-    <mergeCell ref="B2:E2"/>
-    <mergeCell ref="F2:I2"/>
-    <mergeCell ref="J2:M2"/>
-    <mergeCell ref="N2:Q2"/>
-    <mergeCell ref="R2:U2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>

</xml_diff>